<commit_message>
Store Total Duration as plain text values instead of formulas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWgGHmypEGkWY9TAKKf2HP
</commit_message>
<xml_diff>
--- a/output/sept_office.xlsx
+++ b/output/sept_office.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$G$384</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1" calcId="191029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2459,9 +2459,10 @@
       <c r="F40" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="G40" s="79">
-        <f>HOUR(F40-E40)+MINUTE(F40-E40)/100</f>
-        <v>3.23</v>
+      <c r="G40" s="79" t="inlineStr">
+        <is>
+          <t>3.23</t>
+        </is>
       </c>
     </row>
     <row r="41" spans="1:7" ht="14.25" customHeight="1">
@@ -2483,9 +2484,10 @@
       <c r="F41" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="79">
-        <f>HOUR(F41-E41)+MINUTE(F41-E41)/100</f>
-        <v>7.45</v>
+      <c r="G41" s="79" t="inlineStr">
+        <is>
+          <t>7.45</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:7" ht="14.25" customHeight="1">
@@ -2507,9 +2509,10 @@
       <c r="F42" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="79">
-        <f>HOUR(F42-E42)+MINUTE(F42-E42)/100</f>
-        <v>1.45</v>
+      <c r="G42" s="79" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
       </c>
     </row>
     <row r="43" spans="1:7" ht="14.25" customHeight="1">
@@ -2577,9 +2580,10 @@
       <c r="F45" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G45" s="79">
-        <f>HOUR(F45-E45)+MINUTE(F45-E45)/100</f>
-        <v>4.35</v>
+      <c r="G45" s="79" t="inlineStr">
+        <is>
+          <t>4.35</t>
+        </is>
       </c>
     </row>
     <row r="46" spans="1:7" ht="14.25" customHeight="1">
@@ -2624,9 +2628,10 @@
       <c r="F47" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G47" s="79">
-        <f>HOUR(F47-E47)+MINUTE(F47-E47)/100</f>
-        <v>9.1</v>
+      <c r="G47" s="79" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="48" spans="1:7" ht="14.25" customHeight="1">
@@ -2648,9 +2653,10 @@
       <c r="F48" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G48" s="79">
-        <f>HOUR(F48-E48)+MINUTE(F48-E48)/100</f>
-        <v>9.07</v>
+      <c r="G48" s="79" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="49" spans="1:7" ht="14.25" customHeight="1">
@@ -2672,9 +2678,10 @@
       <c r="F49" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G49" s="79">
-        <f>HOUR(F49-E49)+MINUTE(F49-E49)/100</f>
-        <v>9.07</v>
+      <c r="G49" s="79" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="50" spans="1:7" ht="14.25" customHeight="1">
@@ -2719,9 +2726,10 @@
       <c r="F51" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G51" s="79">
-        <f>HOUR(F51-E51)+MINUTE(F51-E51)/100</f>
-        <v>9.17</v>
+      <c r="G51" s="79" t="inlineStr">
+        <is>
+          <t>9.17</t>
+        </is>
       </c>
     </row>
     <row r="52" spans="1:7" ht="14.25" customHeight="1">
@@ -2743,9 +2751,10 @@
       <c r="F52" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G52" s="79">
-        <f>HOUR(F52-E52)+MINUTE(F52-E52)/100</f>
-        <v>9.13</v>
+      <c r="G52" s="79" t="inlineStr">
+        <is>
+          <t>9.13</t>
+        </is>
       </c>
     </row>
     <row r="53" spans="1:7" ht="14.25" customHeight="1">
@@ -2767,9 +2776,10 @@
       <c r="F53" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G53" s="79">
-        <f>HOUR(F53-E53)+MINUTE(F53-E53)/100</f>
-        <v>9.16</v>
+      <c r="G53" s="79" t="inlineStr">
+        <is>
+          <t>9.16</t>
+        </is>
       </c>
     </row>
     <row r="54" spans="1:7" ht="14.25" customHeight="1">
@@ -2791,9 +2801,10 @@
       <c r="F54" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G54" s="79">
-        <f>HOUR(F54-E54)+MINUTE(F54-E54)/100</f>
-        <v>9.09</v>
+      <c r="G54" s="79" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="55" spans="1:7" ht="14.25" customHeight="1">
@@ -2815,9 +2826,10 @@
       <c r="F55" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="G55" s="79">
-        <f>HOUR(F55-E55)+MINUTE(F55-E55)/100</f>
-        <v>9.08</v>
+      <c r="G55" s="79" t="inlineStr">
+        <is>
+          <t>9.08</t>
+        </is>
       </c>
     </row>
     <row r="56" spans="1:7" ht="14.25" customHeight="1">
@@ -2839,9 +2851,10 @@
       <c r="F56" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G56" s="79">
-        <f>HOUR(F56-E56)+MINUTE(F56-E56)/100</f>
-        <v>9.19</v>
+      <c r="G56" s="79" t="inlineStr">
+        <is>
+          <t>9.19</t>
+        </is>
       </c>
     </row>
     <row r="57" spans="1:7" ht="14.25" customHeight="1">
@@ -2886,9 +2899,10 @@
       <c r="F58" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G58" s="79">
-        <f>HOUR(F58-E58)+MINUTE(F58-E58)/100</f>
-        <v>9.08</v>
+      <c r="G58" s="79" t="inlineStr">
+        <is>
+          <t>9.08</t>
+        </is>
       </c>
     </row>
     <row r="59" spans="1:7" ht="14.25" customHeight="1">
@@ -2910,9 +2924,10 @@
       <c r="F59" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G59" s="79">
-        <f>HOUR(F59-E59)+MINUTE(F59-E59)/100</f>
-        <v>9.17</v>
+      <c r="G59" s="79" t="inlineStr">
+        <is>
+          <t>9.17</t>
+        </is>
       </c>
     </row>
     <row r="60" spans="1:7" ht="14.25" customHeight="1">
@@ -2957,9 +2972,10 @@
       <c r="F61" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G61" s="79">
-        <f>HOUR(F61-E61)+MINUTE(F61-E61)/100</f>
-        <v>1.3</v>
+      <c r="G61" s="79" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
       </c>
     </row>
     <row r="62" spans="1:7" ht="14.25" customHeight="1">
@@ -3004,9 +3020,10 @@
       <c r="F63" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G63" s="79">
-        <f>HOUR(F63-E63)+MINUTE(F63-E63)/100</f>
-        <v>8.58</v>
+      <c r="G63" s="79" t="inlineStr">
+        <is>
+          <t>8.58</t>
+        </is>
       </c>
     </row>
     <row r="64" spans="1:7" ht="14.25" customHeight="1">
@@ -3051,9 +3068,10 @@
       <c r="F65" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G65" s="79">
-        <f>HOUR(F65-E65)+MINUTE(F65-E65)/100</f>
-        <v>9.09</v>
+      <c r="G65" s="79" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="66" spans="1:7" ht="14.25" customHeight="1">
@@ -3075,9 +3093,10 @@
       <c r="F66" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G66" s="79">
-        <f>HOUR(F66-E66)+MINUTE(F66-E66)/100</f>
-        <v>9.13</v>
+      <c r="G66" s="79" t="inlineStr">
+        <is>
+          <t>9.13</t>
+        </is>
       </c>
     </row>
     <row r="67" spans="1:7" ht="14.25" customHeight="1">
@@ -3099,9 +3118,10 @@
       <c r="F67" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G67" s="79">
-        <f>HOUR(F67-E67)+MINUTE(F67-E67)/100</f>
-        <v>9.04</v>
+      <c r="G67" s="79" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
       </c>
     </row>
     <row r="68" spans="1:7" ht="14.25" customHeight="1">
@@ -3123,9 +3143,10 @@
       <c r="F68" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G68" s="79">
-        <f>HOUR(F68-E68)+MINUTE(F68-E68)/100</f>
-        <v>8.59</v>
+      <c r="G68" s="79" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
       </c>
     </row>
     <row r="69" spans="1:7" ht="14.25" customHeight="1">
@@ -3147,9 +3168,10 @@
       <c r="F69" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G69" s="79">
-        <f>HOUR(F69-E69)+MINUTE(F69-E69)/100</f>
-        <v>9.1</v>
+      <c r="G69" s="79" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="70" spans="1:7" ht="14.25" customHeight="1">
@@ -3443,9 +3465,10 @@
       <c r="F86" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G86" s="80">
-        <f>HOUR(F86-E86)+MINUTE(F86-E86)/100</f>
-        <v>9.25</v>
+      <c r="G86" s="80" t="inlineStr">
+        <is>
+          <t>9.25</t>
+        </is>
       </c>
     </row>
     <row r="87" spans="1:7" ht="14.25" customHeight="1">
@@ -3467,9 +3490,10 @@
       <c r="F87" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="G87" s="80">
-        <f>HOUR(F87-E87)+MINUTE(F87-E87)/100</f>
-        <v>8.32</v>
+      <c r="G87" s="80" t="inlineStr">
+        <is>
+          <t>8.32</t>
+        </is>
       </c>
     </row>
     <row r="88" spans="1:7" ht="14.25" customHeight="1">
@@ -3514,9 +3538,10 @@
       <c r="F89" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="G89" s="80">
-        <f>HOUR(F89-E89)+MINUTE(F89-E89)/100</f>
-        <v>8.46</v>
+      <c r="G89" s="80" t="inlineStr">
+        <is>
+          <t>8.46</t>
+        </is>
       </c>
     </row>
     <row r="90" spans="1:7" ht="14.25" customHeight="1">
@@ -3538,9 +3563,10 @@
       <c r="F90" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G90" s="80">
-        <f>HOUR(F90-E90)+MINUTE(F90-E90)/100</f>
-        <v>7.54</v>
+      <c r="G90" s="80" t="inlineStr">
+        <is>
+          <t>7.54</t>
+        </is>
       </c>
     </row>
     <row r="91" spans="1:7" ht="14.25" customHeight="1">
@@ -3585,9 +3611,10 @@
       <c r="F92" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="G92" s="80">
-        <f>HOUR(F92-E92)+MINUTE(F92-E92)/100</f>
-        <v>1.56</v>
+      <c r="G92" s="80" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
       </c>
     </row>
     <row r="93" spans="1:7" ht="14.25" customHeight="1">
@@ -3678,9 +3705,10 @@
       <c r="F96" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="G96" s="80">
-        <f>HOUR(F96-E96)+MINUTE(F96-E96)/100</f>
-        <v>8.56</v>
+      <c r="G96" s="80" t="inlineStr">
+        <is>
+          <t>8.56</t>
+        </is>
       </c>
     </row>
     <row r="97" spans="1:7" ht="14.25" customHeight="1">
@@ -3702,9 +3730,10 @@
       <c r="F97" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="G97" s="80">
-        <f>HOUR(F97-E97)+MINUTE(F97-E97)/100</f>
-        <v>3.49</v>
+      <c r="G97" s="80" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
       </c>
     </row>
     <row r="98" spans="1:7" ht="14.25" customHeight="1">
@@ -3726,9 +3755,10 @@
       <c r="F98" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="G98" s="80">
-        <f>HOUR(F98-E98)+MINUTE(F98-E98)/100</f>
-        <v>3.15</v>
+      <c r="G98" s="80" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
       </c>
     </row>
     <row r="99" spans="1:7" ht="14.25" customHeight="1">
@@ -3750,9 +3780,10 @@
       <c r="F99" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="G99" s="80">
-        <f>HOUR(F99-E99)+MINUTE(F99-E99)/100</f>
-        <v>4.26</v>
+      <c r="G99" s="80" t="inlineStr">
+        <is>
+          <t>4.26</t>
+        </is>
       </c>
     </row>
     <row r="100" spans="1:7" ht="14.25" customHeight="1">
@@ -3829,9 +3860,10 @@
       <c r="F103" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G103" s="80">
-        <f>HOUR(F103-E103)+MINUTE(F103-E103)/100</f>
-        <v>6.46</v>
+      <c r="G103" s="80" t="inlineStr">
+        <is>
+          <t>6.46</t>
+        </is>
       </c>
     </row>
     <row r="104" spans="1:7" ht="14.25" customHeight="1">
@@ -3853,9 +3885,10 @@
       <c r="F104" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="G104" s="80">
-        <f>HOUR(F104-E104)+MINUTE(F104-E104)/100</f>
-        <v>2.07</v>
+      <c r="G104" s="80" t="inlineStr">
+        <is>
+          <t>2.07</t>
+        </is>
       </c>
     </row>
     <row r="105" spans="1:7" ht="14.25" customHeight="1">
@@ -3923,9 +3956,10 @@
       <c r="F107" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G107" s="80">
-        <f>HOUR(F107-E107)+MINUTE(F107-E107)/100</f>
-        <v>4.34</v>
+      <c r="G107" s="80" t="inlineStr">
+        <is>
+          <t>4.34</t>
+        </is>
       </c>
     </row>
     <row r="108" spans="1:7" ht="14.25" customHeight="1">
@@ -3970,9 +4004,10 @@
       <c r="F109" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G109" s="80">
-        <f>HOUR(F109-E109)+MINUTE(F109-E109)/100</f>
-        <v>9.09</v>
+      <c r="G109" s="80" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="110" spans="1:7" ht="14.25" customHeight="1">
@@ -3994,9 +4029,10 @@
       <c r="F110" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G110" s="80">
-        <f>HOUR(F110-E110)+MINUTE(F110-E110)/100</f>
-        <v>9.06</v>
+      <c r="G110" s="80" t="inlineStr">
+        <is>
+          <t>9.06</t>
+        </is>
       </c>
     </row>
     <row r="111" spans="1:7" ht="14.25" customHeight="1">
@@ -4018,9 +4054,10 @@
       <c r="F111" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G111" s="80">
-        <f>HOUR(F111-E111)+MINUTE(F111-E111)/100</f>
-        <v>9.07</v>
+      <c r="G111" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="112" spans="1:7" ht="14.25" customHeight="1">
@@ -4065,9 +4102,10 @@
       <c r="F113" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G113" s="80">
-        <f>HOUR(F113-E113)+MINUTE(F113-E113)/100</f>
-        <v>9.09</v>
+      <c r="G113" s="80" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="114" spans="1:7" ht="14.25" customHeight="1">
@@ -4089,9 +4127,10 @@
       <c r="F114" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G114" s="80">
-        <f>HOUR(F114-E114)+MINUTE(F114-E114)/100</f>
-        <v>9.12</v>
+      <c r="G114" s="80" t="inlineStr">
+        <is>
+          <t>9.12</t>
+        </is>
       </c>
     </row>
     <row r="115" spans="1:7" ht="14.25" customHeight="1">
@@ -4113,9 +4152,10 @@
       <c r="F115" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G115" s="80">
-        <f>HOUR(F115-E115)+MINUTE(F115-E115)/100</f>
-        <v>9.14</v>
+      <c r="G115" s="80" t="inlineStr">
+        <is>
+          <t>9.14</t>
+        </is>
       </c>
     </row>
     <row r="116" spans="1:7" ht="14.25" customHeight="1">
@@ -4137,9 +4177,10 @@
       <c r="F116" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G116" s="80">
-        <f>HOUR(F116-E116)+MINUTE(F116-E116)/100</f>
-        <v>9.08</v>
+      <c r="G116" s="80" t="inlineStr">
+        <is>
+          <t>9.08</t>
+        </is>
       </c>
     </row>
     <row r="117" spans="1:7" ht="14.25" customHeight="1">
@@ -4161,9 +4202,10 @@
       <c r="F117" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G117" s="80">
-        <f>HOUR(F117-E117)+MINUTE(F117-E117)/100</f>
-        <v>9</v>
+      <c r="G117" s="80" t="inlineStr">
+        <is>
+          <t>9.00</t>
+        </is>
       </c>
     </row>
     <row r="118" spans="1:7" ht="14.25" customHeight="1">
@@ -4185,9 +4227,10 @@
       <c r="F118" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G118" s="80">
-        <f>HOUR(F118-E118)+MINUTE(F118-E118)/100</f>
-        <v>9.18</v>
+      <c r="G118" s="80" t="inlineStr">
+        <is>
+          <t>9.18</t>
+        </is>
       </c>
     </row>
     <row r="119" spans="1:7" ht="14.25" customHeight="1">
@@ -4232,9 +4275,10 @@
       <c r="F120" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G120" s="80">
-        <f>HOUR(F120-E120)+MINUTE(F120-E120)/100</f>
-        <v>9.06</v>
+      <c r="G120" s="80" t="inlineStr">
+        <is>
+          <t>9.06</t>
+        </is>
       </c>
     </row>
     <row r="121" spans="1:7" ht="14.25" customHeight="1">
@@ -4256,9 +4300,10 @@
       <c r="F121" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G121" s="80">
-        <f>HOUR(F121-E121)+MINUTE(F121-E121)/100</f>
-        <v>8.59</v>
+      <c r="G121" s="80" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
       </c>
     </row>
     <row r="122" spans="1:7" ht="14.25" customHeight="1">
@@ -4280,9 +4325,10 @@
       <c r="F122" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G122" s="80">
-        <f>HOUR(F122-E122)+MINUTE(F122-E122)/100</f>
-        <v>8.52</v>
+      <c r="G122" s="80" t="inlineStr">
+        <is>
+          <t>8.52</t>
+        </is>
       </c>
     </row>
     <row r="123" spans="1:7" ht="14.25" customHeight="1">
@@ -4304,9 +4350,10 @@
       <c r="F123" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G123" s="80">
-        <f>HOUR(F123-E123)+MINUTE(F123-E123)/100</f>
-        <v>1.36</v>
+      <c r="G123" s="80" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
       </c>
     </row>
     <row r="124" spans="1:7" ht="14.25" customHeight="1">
@@ -4351,9 +4398,10 @@
       <c r="F125" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G125" s="80">
-        <f>HOUR(F125-E125)+MINUTE(F125-E125)/100</f>
-        <v>8.16</v>
+      <c r="G125" s="80" t="inlineStr">
+        <is>
+          <t>8.16</t>
+        </is>
       </c>
     </row>
     <row r="126" spans="1:7" ht="14.25" customHeight="1">
@@ -4398,9 +4446,10 @@
       <c r="F127" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G127" s="80">
-        <f>HOUR(F127-E127)+MINUTE(F127-E127)/100</f>
-        <v>9.07</v>
+      <c r="G127" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="128" spans="1:7" ht="14.25" customHeight="1">
@@ -4422,9 +4471,10 @@
       <c r="F128" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G128" s="80">
-        <f>HOUR(F128-E128)+MINUTE(F128-E128)/100</f>
-        <v>9.04</v>
+      <c r="G128" s="80" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
       </c>
     </row>
     <row r="129" spans="1:7" ht="14.25" customHeight="1">
@@ -4446,9 +4496,10 @@
       <c r="F129" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G129" s="80">
-        <f>HOUR(F129-E129)+MINUTE(F129-E129)/100</f>
-        <v>8.5</v>
+      <c r="G129" s="80" t="inlineStr">
+        <is>
+          <t>8.50</t>
+        </is>
       </c>
     </row>
     <row r="130" spans="1:7" ht="14.25" customHeight="1">
@@ -4470,9 +4521,10 @@
       <c r="F130" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G130" s="80">
-        <f>HOUR(F130-E130)+MINUTE(F130-E130)/100</f>
-        <v>8.54</v>
+      <c r="G130" s="80" t="inlineStr">
+        <is>
+          <t>8.54</t>
+        </is>
       </c>
     </row>
     <row r="131" spans="1:7" ht="14.25" customHeight="1">
@@ -4494,9 +4546,10 @@
       <c r="F131" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G131" s="80">
-        <f>HOUR(F131-E131)+MINUTE(F131-E131)/100</f>
-        <v>9.12</v>
+      <c r="G131" s="80" t="inlineStr">
+        <is>
+          <t>9.12</t>
+        </is>
       </c>
     </row>
     <row r="132" spans="1:7" ht="14.25" customHeight="1">
@@ -4550,9 +4603,10 @@
       <c r="F134" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="G134" s="80">
-        <f>HOUR(F134-E134)+MINUTE(F134-E134)/100</f>
-        <v>7.41</v>
+      <c r="G134" s="80" t="inlineStr">
+        <is>
+          <t>7.41</t>
+        </is>
       </c>
     </row>
     <row r="135" spans="1:7" ht="14.25" customHeight="1">
@@ -4643,9 +4697,10 @@
       <c r="F138" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="G138" s="80">
-        <f>HOUR(F138-E138)+MINUTE(F138-E138)/100</f>
-        <v>2.23</v>
+      <c r="G138" s="80" t="inlineStr">
+        <is>
+          <t>2.23</t>
+        </is>
       </c>
     </row>
     <row r="139" spans="1:7" ht="14.25" customHeight="1">
@@ -4690,9 +4745,10 @@
       <c r="F140" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="G140" s="80">
-        <f>HOUR(F140-E140)+MINUTE(F140-E140)/100</f>
-        <v>7.47</v>
+      <c r="G140" s="80" t="inlineStr">
+        <is>
+          <t>7.47</t>
+        </is>
       </c>
     </row>
     <row r="141" spans="1:7" ht="14.25" customHeight="1">
@@ -4737,9 +4793,10 @@
       <c r="F142" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="G142" s="80">
-        <f>HOUR(F142-E142)+MINUTE(F142-E142)/100</f>
-        <v>8.04</v>
+      <c r="G142" s="80" t="inlineStr">
+        <is>
+          <t>8.04</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:7" ht="14.25" customHeight="1">
@@ -4807,9 +4864,10 @@
       <c r="F145" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G145" s="80">
-        <f>HOUR(F145-E145)+MINUTE(F145-E145)/100</f>
-        <v>7.45</v>
+      <c r="G145" s="80" t="inlineStr">
+        <is>
+          <t>7.45</t>
+        </is>
       </c>
     </row>
     <row r="146" spans="1:7" ht="14.25" customHeight="1">
@@ -4831,9 +4889,10 @@
       <c r="F146" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="G146" s="80">
-        <f>HOUR(F146-E146)+MINUTE(F146-E146)/100</f>
-        <v>7.52</v>
+      <c r="G146" s="80" t="inlineStr">
+        <is>
+          <t>7.52</t>
+        </is>
       </c>
     </row>
     <row r="147" spans="1:7" ht="14.25" customHeight="1">
@@ -4855,9 +4914,10 @@
       <c r="F147" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="G147" s="80">
-        <f>HOUR(F147-E147)+MINUTE(F147-E147)/100</f>
-        <v>7.58</v>
+      <c r="G147" s="80" t="inlineStr">
+        <is>
+          <t>7.58</t>
+        </is>
       </c>
     </row>
     <row r="148" spans="1:7" ht="14.25" customHeight="1">
@@ -4879,9 +4939,10 @@
       <c r="F148" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="G148" s="80">
-        <f>HOUR(F148-E148)+MINUTE(F148-E148)/100</f>
-        <v>7.53</v>
+      <c r="G148" s="80" t="inlineStr">
+        <is>
+          <t>7.53</t>
+        </is>
       </c>
     </row>
     <row r="149" spans="1:7" ht="14.25" customHeight="1">
@@ -4903,9 +4964,10 @@
       <c r="F149" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="G149" s="80">
-        <f>HOUR(F149-E149)+MINUTE(F149-E149)/100</f>
-        <v>7.22</v>
+      <c r="G149" s="80" t="inlineStr">
+        <is>
+          <t>7.22</t>
+        </is>
       </c>
     </row>
     <row r="150" spans="1:7" ht="14.25" customHeight="1">
@@ -4973,9 +5035,10 @@
       <c r="F152" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="G152" s="80">
-        <f>HOUR(F152-E152)+MINUTE(F152-E152)/100</f>
-        <v>7.12</v>
+      <c r="G152" s="80" t="inlineStr">
+        <is>
+          <t>7.12</t>
+        </is>
       </c>
     </row>
     <row r="153" spans="1:7" ht="14.25" customHeight="1">
@@ -5020,9 +5083,10 @@
       <c r="F154" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="G154" s="80">
-        <f>HOUR(F154-E154)+MINUTE(F154-E154)/100</f>
-        <v>0.5</v>
+      <c r="G154" s="80" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
       </c>
     </row>
     <row r="155" spans="1:7" ht="14.25" customHeight="1">
@@ -5136,9 +5200,10 @@
       <c r="F159" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="G159" s="80">
-        <f>HOUR(F159-E159)+MINUTE(F159-E159)/100</f>
-        <v>8.01</v>
+      <c r="G159" s="80" t="inlineStr">
+        <is>
+          <t>8.01</t>
+        </is>
       </c>
     </row>
     <row r="160" spans="1:7" ht="14.25" customHeight="1">
@@ -5160,9 +5225,10 @@
       <c r="F160" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="G160" s="80">
-        <f>HOUR(F160-E160)+MINUTE(F160-E160)/100</f>
-        <v>7.54</v>
+      <c r="G160" s="80" t="inlineStr">
+        <is>
+          <t>7.54</t>
+        </is>
       </c>
     </row>
     <row r="161" spans="1:7" ht="14.25" customHeight="1">
@@ -5184,9 +5250,10 @@
       <c r="F161" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="G161" s="80">
-        <f>HOUR(F161-E161)+MINUTE(F161-E161)/100</f>
-        <v>7.58</v>
+      <c r="G161" s="80" t="inlineStr">
+        <is>
+          <t>7.58</t>
+        </is>
       </c>
     </row>
     <row r="162" spans="1:7" ht="14.25" customHeight="1">
@@ -5208,9 +5275,10 @@
       <c r="F162" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="G162" s="80">
-        <f>HOUR(F162-E162)+MINUTE(F162-E162)/100</f>
-        <v>7.31</v>
+      <c r="G162" s="80" t="inlineStr">
+        <is>
+          <t>7.31</t>
+        </is>
       </c>
     </row>
     <row r="163" spans="1:7" ht="14.25" customHeight="1">
@@ -5241,9 +5309,10 @@
       <c r="F164" s="23">
         <v>0.73958333333333337</v>
       </c>
-      <c r="G164" s="80">
-        <f>HOUR(F164-E164)+MINUTE(F164-E164)/100</f>
-        <v>9.27</v>
+      <c r="G164" s="80" t="inlineStr">
+        <is>
+          <t>9.27</t>
+        </is>
       </c>
     </row>
     <row r="165" spans="1:7" ht="14.25" customHeight="1">
@@ -5265,9 +5334,10 @@
       <c r="F165" s="23">
         <v>0.75</v>
       </c>
-      <c r="G165" s="80">
-        <f>HOUR(F165-E165)+MINUTE(F165-E165)/100</f>
-        <v>8.54</v>
+      <c r="G165" s="80" t="inlineStr">
+        <is>
+          <t>8.54</t>
+        </is>
       </c>
     </row>
     <row r="166" spans="1:7" ht="14.25" customHeight="1">
@@ -5289,9 +5359,10 @@
       <c r="F166" s="23">
         <v>0.81041666666666667</v>
       </c>
-      <c r="G166" s="80">
-        <f>HOUR(F166-E166)+MINUTE(F166-E166)/100</f>
-        <v>11.02</v>
+      <c r="G166" s="80" t="inlineStr">
+        <is>
+          <t>11.02</t>
+        </is>
       </c>
     </row>
     <row r="167" spans="1:7" ht="14.25" customHeight="1">
@@ -5359,9 +5430,10 @@
       <c r="F169" s="23">
         <v>0.76527777777777772</v>
       </c>
-      <c r="G169" s="80">
-        <f>HOUR(F169-E169)+MINUTE(F169-E169)/100</f>
-        <v>9.37</v>
+      <c r="G169" s="80" t="inlineStr">
+        <is>
+          <t>9.37</t>
+        </is>
       </c>
     </row>
     <row r="170" spans="1:7" ht="14.25" customHeight="1">
@@ -5406,9 +5478,10 @@
       <c r="F171" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="G171" s="80">
-        <f>HOUR(F171-E171)+MINUTE(F171-E171)/100</f>
-        <v>6.44</v>
+      <c r="G171" s="80" t="inlineStr">
+        <is>
+          <t>6.44</t>
+        </is>
       </c>
     </row>
     <row r="172" spans="1:7" ht="14.25" customHeight="1">
@@ -5430,9 +5503,10 @@
       <c r="F172" s="23">
         <v>0.92638888888888893</v>
       </c>
-      <c r="G172" s="80">
-        <f>HOUR(F172-E172)+MINUTE(F172-E172)/100</f>
-        <v>13.32</v>
+      <c r="G172" s="80" t="inlineStr">
+        <is>
+          <t>13.32</t>
+        </is>
       </c>
     </row>
     <row r="173" spans="1:7" ht="14.25" customHeight="1">
@@ -5454,9 +5528,10 @@
       <c r="F173" s="23">
         <v>0.7368055555555556</v>
       </c>
-      <c r="G173" s="80">
-        <f>HOUR(F173-E173)+MINUTE(F173-E173)/100</f>
-        <v>9.36</v>
+      <c r="G173" s="80" t="inlineStr">
+        <is>
+          <t>9.36</t>
+        </is>
       </c>
     </row>
     <row r="174" spans="1:7" ht="14.25" customHeight="1">
@@ -5501,9 +5576,10 @@
       <c r="F175" s="23">
         <v>0.75624999999999998</v>
       </c>
-      <c r="G175" s="80">
-        <f>HOUR(F175-E175)+MINUTE(F175-E175)/100</f>
-        <v>9.41</v>
+      <c r="G175" s="80" t="inlineStr">
+        <is>
+          <t>9.41</t>
+        </is>
       </c>
     </row>
     <row r="176" spans="1:7" ht="14.25" customHeight="1">
@@ -5525,9 +5601,10 @@
       <c r="F176" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G176" s="80">
-        <f>HOUR(F176-E176)+MINUTE(F176-E176)/100</f>
-        <v>8.48</v>
+      <c r="G176" s="80" t="inlineStr">
+        <is>
+          <t>8.48</t>
+        </is>
       </c>
     </row>
     <row r="177" spans="1:7" ht="14.25" customHeight="1">
@@ -5549,9 +5626,10 @@
       <c r="F177" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="G177" s="80">
-        <f>HOUR(F177-E177)+MINUTE(F177-E177)/100</f>
-        <v>8.52</v>
+      <c r="G177" s="80" t="inlineStr">
+        <is>
+          <t>8.52</t>
+        </is>
       </c>
     </row>
     <row r="178" spans="1:7" ht="14.25" customHeight="1">
@@ -5573,9 +5651,10 @@
       <c r="F178" s="23">
         <v>0.91805555555555551</v>
       </c>
-      <c r="G178" s="80">
-        <f>HOUR(F178-E178)+MINUTE(F178-E178)/100</f>
-        <v>12.56</v>
+      <c r="G178" s="80" t="inlineStr">
+        <is>
+          <t>12.56</t>
+        </is>
       </c>
     </row>
     <row r="179" spans="1:7" ht="14.25" customHeight="1">
@@ -5597,9 +5676,10 @@
       <c r="F179" s="23">
         <v>0.80347222222222225</v>
       </c>
-      <c r="G179" s="80">
-        <f>HOUR(F179-E179)+MINUTE(F179-E179)/100</f>
-        <v>10.58</v>
+      <c r="G179" s="80" t="inlineStr">
+        <is>
+          <t>10.58</t>
+        </is>
       </c>
     </row>
     <row r="180" spans="1:7" ht="14.25" customHeight="1">
@@ -5621,9 +5701,10 @@
       <c r="F180" s="23">
         <v>0.7416666666666667</v>
       </c>
-      <c r="G180" s="80">
-        <f>HOUR(F180-E180)+MINUTE(F180-E180)/100</f>
-        <v>9.09</v>
+      <c r="G180" s="80" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="181" spans="1:7" ht="14.25" customHeight="1">
@@ -5668,9 +5749,10 @@
       <c r="F182" s="23">
         <v>0.87152777777777779</v>
       </c>
-      <c r="G182" s="80">
-        <f>HOUR(F182-E182)+MINUTE(F182-E182)/100</f>
-        <v>12.11</v>
+      <c r="G182" s="80" t="inlineStr">
+        <is>
+          <t>12.11</t>
+        </is>
       </c>
     </row>
     <row r="183" spans="1:7" ht="14.25" customHeight="1">
@@ -5692,9 +5774,10 @@
       <c r="F183" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="G183" s="80">
-        <f>HOUR(F183-E183)+MINUTE(F183-E183)/100</f>
-        <v>9.38</v>
+      <c r="G183" s="80" t="inlineStr">
+        <is>
+          <t>9.38</t>
+        </is>
       </c>
     </row>
     <row r="184" spans="1:7" ht="14.25" customHeight="1">
@@ -5739,9 +5822,10 @@
       <c r="F185" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="G185" s="80">
-        <f>HOUR(F185-E185)+MINUTE(F185-E185)/100</f>
-        <v>9.44</v>
+      <c r="G185" s="80" t="inlineStr">
+        <is>
+          <t>9.44</t>
+        </is>
       </c>
     </row>
     <row r="186" spans="1:7" ht="14.25" customHeight="1">
@@ -5786,9 +5870,10 @@
       <c r="F187" s="23">
         <v>0.72499999999999998</v>
       </c>
-      <c r="G187" s="80">
-        <f>HOUR(F187-E187)+MINUTE(F187-E187)/100</f>
-        <v>9.19</v>
+      <c r="G187" s="80" t="inlineStr">
+        <is>
+          <t>9.19</t>
+        </is>
       </c>
     </row>
     <row r="188" spans="1:7" ht="14.25" customHeight="1">
@@ -5833,9 +5918,10 @@
       <c r="F189" s="23">
         <v>0.66666666666666663</v>
       </c>
-      <c r="G189" s="80">
-        <f>HOUR(F189-E189)+MINUTE(F189-E189)/100</f>
-        <v>7.17</v>
+      <c r="G189" s="80" t="inlineStr">
+        <is>
+          <t>7.17</t>
+        </is>
       </c>
     </row>
     <row r="190" spans="1:7" ht="14.25" customHeight="1">
@@ -5857,9 +5943,10 @@
       <c r="F190" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="G190" s="80">
-        <f>HOUR(F190-E190)+MINUTE(F190-E190)/100</f>
-        <v>9.26</v>
+      <c r="G190" s="80" t="inlineStr">
+        <is>
+          <t>9.26</t>
+        </is>
       </c>
     </row>
     <row r="191" spans="1:7" ht="14.25" customHeight="1">
@@ -5881,9 +5968,10 @@
       <c r="F191" s="23">
         <v>0.69513888888888886</v>
       </c>
-      <c r="G191" s="80">
-        <f>HOUR(F191-E191)+MINUTE(F191-E191)/100</f>
-        <v>8</v>
+      <c r="G191" s="80" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
       </c>
     </row>
     <row r="192" spans="1:7" ht="14.25" customHeight="1">
@@ -5905,9 +5993,10 @@
       <c r="F192" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G192" s="80">
-        <f>HOUR(F192-E192)+MINUTE(F192-E192)/100</f>
-        <v>8.35</v>
+      <c r="G192" s="80" t="inlineStr">
+        <is>
+          <t>8.35</t>
+        </is>
       </c>
     </row>
     <row r="193" spans="1:7" ht="14.25" customHeight="1">
@@ -5929,9 +6018,10 @@
       <c r="F193" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="G193" s="80">
-        <f>HOUR(F193-E193)+MINUTE(F193-E193)/100</f>
-        <v>9.05</v>
+      <c r="G193" s="80" t="inlineStr">
+        <is>
+          <t>9.05</t>
+        </is>
       </c>
     </row>
     <row r="194" spans="1:7" ht="14.25" customHeight="1">
@@ -6100,9 +6190,10 @@
       <c r="F203" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="G203" s="80">
-        <f>HOUR(F203-E203)+MINUTE(F203-E203)/100</f>
-        <v>2.16</v>
+      <c r="G203" s="80" t="inlineStr">
+        <is>
+          <t>2.16</t>
+        </is>
       </c>
     </row>
     <row r="204" spans="1:7" ht="14.25" customHeight="1">
@@ -6124,9 +6215,10 @@
       <c r="F204" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G204" s="80">
-        <f>HOUR(F204-E204)+MINUTE(F204-E204)/100</f>
-        <v>8.57</v>
+      <c r="G204" s="80" t="inlineStr">
+        <is>
+          <t>8.57</t>
+        </is>
       </c>
     </row>
     <row r="205" spans="1:7" ht="14.25" customHeight="1">
@@ -6171,9 +6263,10 @@
       <c r="F206" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="G206" s="80">
-        <f>HOUR(F206-E206)+MINUTE(F206-E206)/100</f>
-        <v>9.35</v>
+      <c r="G206" s="80" t="inlineStr">
+        <is>
+          <t>9.35</t>
+        </is>
       </c>
     </row>
     <row r="207" spans="1:7" ht="14.25" customHeight="1">
@@ -6195,9 +6288,10 @@
       <c r="F207" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="G207" s="80">
-        <f>HOUR(F207-E207)+MINUTE(F207-E207)/100</f>
-        <v>8.31</v>
+      <c r="G207" s="80" t="inlineStr">
+        <is>
+          <t>8.31</t>
+        </is>
       </c>
     </row>
     <row r="208" spans="1:7" ht="14.25" customHeight="1">
@@ -6219,9 +6313,10 @@
       <c r="F208" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G208" s="80">
-        <f>HOUR(F208-E208)+MINUTE(F208-E208)/100</f>
-        <v>9.03</v>
+      <c r="G208" s="80" t="inlineStr">
+        <is>
+          <t>9.03</t>
+        </is>
       </c>
     </row>
     <row r="209" spans="1:7" ht="14.25" customHeight="1">
@@ -6243,9 +6338,10 @@
       <c r="F209" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G209" s="80">
-        <f>HOUR(F209-E209)+MINUTE(F209-E209)/100</f>
-        <v>9.07</v>
+      <c r="G209" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="210" spans="1:7" ht="14.25" customHeight="1">
@@ -6267,9 +6363,10 @@
       <c r="F210" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="G210" s="80">
-        <f>HOUR(F210-E210)+MINUTE(F210-E210)/100</f>
-        <v>5.04</v>
+      <c r="G210" s="80" t="inlineStr">
+        <is>
+          <t>5.04</t>
+        </is>
       </c>
     </row>
     <row r="211" spans="1:7" ht="14.25" customHeight="1">
@@ -6291,9 +6388,10 @@
       <c r="F211" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G211" s="80">
-        <f>HOUR(F211-E211)+MINUTE(F211-E211)/100</f>
-        <v>9.04</v>
+      <c r="G211" s="80" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
       </c>
     </row>
     <row r="212" spans="1:7" ht="14.25" customHeight="1">
@@ -6338,9 +6436,10 @@
       <c r="F213" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G213" s="80">
-        <f>HOUR(F213-E213)+MINUTE(F213-E213)/100</f>
-        <v>9.1</v>
+      <c r="G213" s="80" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="214" spans="1:7" ht="14.25" customHeight="1">
@@ -6362,9 +6461,10 @@
       <c r="F214" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G214" s="80">
-        <f>HOUR(F214-E214)+MINUTE(F214-E214)/100</f>
-        <v>8.59</v>
+      <c r="G214" s="80" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
       </c>
     </row>
     <row r="215" spans="1:7" ht="14.25" customHeight="1">
@@ -6455,9 +6555,10 @@
       <c r="F218" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="G218" s="80">
-        <f>HOUR(F218-E218)+MINUTE(F218-E218)/100</f>
-        <v>9</v>
+      <c r="G218" s="80" t="inlineStr">
+        <is>
+          <t>9.00</t>
+        </is>
       </c>
     </row>
     <row r="219" spans="1:7" ht="14.25" customHeight="1">
@@ -6502,9 +6603,10 @@
       <c r="F220" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G220" s="80">
-        <f>HOUR(F220-E220)+MINUTE(F220-E220)/100</f>
-        <v>5.55</v>
+      <c r="G220" s="80" t="inlineStr">
+        <is>
+          <t>5.55</t>
+        </is>
       </c>
     </row>
     <row r="221" spans="1:7" ht="14.25" customHeight="1">
@@ -6526,9 +6628,10 @@
       <c r="F221" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="G221" s="80">
-        <f>HOUR(F221-E221)+MINUTE(F221-E221)/100</f>
-        <v>5.41</v>
+      <c r="G221" s="80" t="inlineStr">
+        <is>
+          <t>5.41</t>
+        </is>
       </c>
     </row>
     <row r="222" spans="1:7" ht="14.25" customHeight="1">
@@ -6550,9 +6653,10 @@
       <c r="F222" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G222" s="80">
-        <f>HOUR(F222-E222)+MINUTE(F222-E222)/100</f>
-        <v>9.04</v>
+      <c r="G222" s="80" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
       </c>
     </row>
     <row r="223" spans="1:7" ht="14.25" customHeight="1">
@@ -6574,9 +6678,10 @@
       <c r="F223" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G223" s="80">
-        <f>HOUR(F223-E223)+MINUTE(F223-E223)/100</f>
-        <v>8.51</v>
+      <c r="G223" s="80" t="inlineStr">
+        <is>
+          <t>8.51</t>
+        </is>
       </c>
     </row>
     <row r="224" spans="1:7" ht="14.25" customHeight="1">
@@ -6598,9 +6703,10 @@
       <c r="F224" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G224" s="80">
-        <f>HOUR(F224-E224)+MINUTE(F224-E224)/100</f>
-        <v>9.05</v>
+      <c r="G224" s="80" t="inlineStr">
+        <is>
+          <t>9.05</t>
+        </is>
       </c>
     </row>
     <row r="225" spans="1:7" ht="14.25" customHeight="1">
@@ -6631,9 +6737,10 @@
       <c r="F226" s="23">
         <v>0.73958333333333337</v>
       </c>
-      <c r="G226" s="80">
-        <f>HOUR(F226-E226)+MINUTE(F226-E226)/100</f>
-        <v>9.27</v>
+      <c r="G226" s="80" t="inlineStr">
+        <is>
+          <t>9.27</t>
+        </is>
       </c>
     </row>
     <row r="227" spans="1:7" ht="14.25" customHeight="1">
@@ -6655,9 +6762,10 @@
       <c r="F227" s="23">
         <v>0.75</v>
       </c>
-      <c r="G227" s="80">
-        <f>HOUR(F227-E227)+MINUTE(F227-E227)/100</f>
-        <v>8.54</v>
+      <c r="G227" s="80" t="inlineStr">
+        <is>
+          <t>8.54</t>
+        </is>
       </c>
     </row>
     <row r="228" spans="1:7" ht="14.25" customHeight="1">
@@ -6679,9 +6787,10 @@
       <c r="F228" s="23">
         <v>0.81041666666666667</v>
       </c>
-      <c r="G228" s="80">
-        <f>HOUR(F228-E228)+MINUTE(F228-E228)/100</f>
-        <v>11.02</v>
+      <c r="G228" s="80" t="inlineStr">
+        <is>
+          <t>11.02</t>
+        </is>
       </c>
     </row>
     <row r="229" spans="1:7" ht="14.25" customHeight="1">
@@ -6749,9 +6858,10 @@
       <c r="F231" s="78">
         <v>0.76527777777777772</v>
       </c>
-      <c r="G231" s="80">
-        <f>HOUR(F231-E231)+MINUTE(F231-E231)/100</f>
-        <v>9.37</v>
+      <c r="G231" s="80" t="inlineStr">
+        <is>
+          <t>9.37</t>
+        </is>
       </c>
     </row>
     <row r="232" spans="1:7" ht="14.25" customHeight="1">
@@ -6796,9 +6906,10 @@
       <c r="F233" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="G233" s="80">
-        <f>HOUR(F233-E233)+MINUTE(F233-E233)/100</f>
-        <v>6.44</v>
+      <c r="G233" s="80" t="inlineStr">
+        <is>
+          <t>6.44</t>
+        </is>
       </c>
     </row>
     <row r="234" spans="1:7" ht="14.25" customHeight="1">
@@ -6820,9 +6931,10 @@
       <c r="F234" s="78">
         <v>0.92638888888888893</v>
       </c>
-      <c r="G234" s="80">
-        <f>HOUR(F234-E234)+MINUTE(F234-E234)/100</f>
-        <v>13.32</v>
+      <c r="G234" s="80" t="inlineStr">
+        <is>
+          <t>13.32</t>
+        </is>
       </c>
     </row>
     <row r="235" spans="1:7" ht="14.25" customHeight="1">
@@ -6844,9 +6956,10 @@
       <c r="F235" s="23">
         <v>0.7368055555555556</v>
       </c>
-      <c r="G235" s="80">
-        <f>HOUR(F235-E235)+MINUTE(F235-E235)/100</f>
-        <v>9.36</v>
+      <c r="G235" s="80" t="inlineStr">
+        <is>
+          <t>9.36</t>
+        </is>
       </c>
     </row>
     <row r="236" spans="1:7" ht="14.25" customHeight="1">
@@ -6891,9 +7004,10 @@
       <c r="F237" s="23">
         <v>0.75624999999999998</v>
       </c>
-      <c r="G237" s="80">
-        <f>HOUR(F237-E237)+MINUTE(F237-E237)/100</f>
-        <v>9.41</v>
+      <c r="G237" s="80" t="inlineStr">
+        <is>
+          <t>9.41</t>
+        </is>
       </c>
     </row>
     <row r="238" spans="1:7" ht="14.25" customHeight="1">
@@ -6915,9 +7029,10 @@
       <c r="F238" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G238" s="80">
-        <f>HOUR(F238-E238)+MINUTE(F238-E238)/100</f>
-        <v>8.48</v>
+      <c r="G238" s="80" t="inlineStr">
+        <is>
+          <t>8.48</t>
+        </is>
       </c>
     </row>
     <row r="239" spans="1:7" ht="14.25" customHeight="1">
@@ -6939,9 +7054,10 @@
       <c r="F239" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="G239" s="80">
-        <f>HOUR(F239-E239)+MINUTE(F239-E239)/100</f>
-        <v>8.52</v>
+      <c r="G239" s="80" t="inlineStr">
+        <is>
+          <t>8.52</t>
+        </is>
       </c>
     </row>
     <row r="240" spans="1:7" ht="14.25" customHeight="1">
@@ -6963,9 +7079,10 @@
       <c r="F240" s="23">
         <v>0.91805555555555551</v>
       </c>
-      <c r="G240" s="80">
-        <f>HOUR(F240-E240)+MINUTE(F240-E240)/100</f>
-        <v>12.56</v>
+      <c r="G240" s="80" t="inlineStr">
+        <is>
+          <t>12.56</t>
+        </is>
       </c>
     </row>
     <row r="241" spans="1:7" ht="14.25" customHeight="1">
@@ -6987,9 +7104,10 @@
       <c r="F241" s="23">
         <v>0.80347222222222225</v>
       </c>
-      <c r="G241" s="80">
-        <f>HOUR(F241-E241)+MINUTE(F241-E241)/100</f>
-        <v>10.58</v>
+      <c r="G241" s="80" t="inlineStr">
+        <is>
+          <t>10.58</t>
+        </is>
       </c>
     </row>
     <row r="242" spans="1:7" ht="14.25" customHeight="1">
@@ -7011,9 +7129,10 @@
       <c r="F242" s="23">
         <v>0.7416666666666667</v>
       </c>
-      <c r="G242" s="80">
-        <f>HOUR(F242-E242)+MINUTE(F242-E242)/100</f>
-        <v>9.09</v>
+      <c r="G242" s="80" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
       </c>
     </row>
     <row r="243" spans="1:7" ht="14.25" customHeight="1">
@@ -7058,9 +7177,10 @@
       <c r="F244" s="23">
         <v>0.87152777777777779</v>
       </c>
-      <c r="G244" s="80">
-        <f>HOUR(F244-E244)+MINUTE(F244-E244)/100</f>
-        <v>12.11</v>
+      <c r="G244" s="80" t="inlineStr">
+        <is>
+          <t>12.11</t>
+        </is>
       </c>
     </row>
     <row r="245" spans="1:7" ht="14.25" customHeight="1">
@@ -7082,9 +7202,10 @@
       <c r="F245" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="G245" s="80">
-        <f>HOUR(F245-E245)+MINUTE(F245-E245)/100</f>
-        <v>9.38</v>
+      <c r="G245" s="80" t="inlineStr">
+        <is>
+          <t>9.38</t>
+        </is>
       </c>
     </row>
     <row r="246" spans="1:7" ht="14.25" customHeight="1">
@@ -7129,9 +7250,10 @@
       <c r="F247" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="G247" s="80">
-        <f>HOUR(F247-E247)+MINUTE(F247-E247)/100</f>
-        <v>9.44</v>
+      <c r="G247" s="80" t="inlineStr">
+        <is>
+          <t>9.44</t>
+        </is>
       </c>
     </row>
     <row r="248" spans="1:7" ht="14.25" customHeight="1">
@@ -7176,9 +7298,10 @@
       <c r="F249" s="23">
         <v>0.72499999999999998</v>
       </c>
-      <c r="G249" s="80">
-        <f>HOUR(F249-E249)+MINUTE(F249-E249)/100</f>
-        <v>9.19</v>
+      <c r="G249" s="80" t="inlineStr">
+        <is>
+          <t>9.19</t>
+        </is>
       </c>
     </row>
     <row r="250" spans="1:7" ht="14.25" customHeight="1">
@@ -7223,9 +7346,10 @@
       <c r="F251" s="23">
         <v>0.66666666666666663</v>
       </c>
-      <c r="G251" s="80">
-        <f>HOUR(F251-E251)+MINUTE(F251-E251)/100</f>
-        <v>7.17</v>
+      <c r="G251" s="80" t="inlineStr">
+        <is>
+          <t>7.17</t>
+        </is>
       </c>
     </row>
     <row r="252" spans="1:7" ht="14.25" customHeight="1">
@@ -7247,9 +7371,10 @@
       <c r="F252" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="G252" s="80">
-        <f>HOUR(F252-E252)+MINUTE(F252-E252)/100</f>
-        <v>9.26</v>
+      <c r="G252" s="80" t="inlineStr">
+        <is>
+          <t>9.26</t>
+        </is>
       </c>
     </row>
     <row r="253" spans="1:7" ht="14.25" customHeight="1">
@@ -7271,9 +7396,10 @@
       <c r="F253" s="23">
         <v>0.69513888888888886</v>
       </c>
-      <c r="G253" s="80">
-        <f>HOUR(F253-E253)+MINUTE(F253-E253)/100</f>
-        <v>8</v>
+      <c r="G253" s="80" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
       </c>
     </row>
     <row r="254" spans="1:7" ht="14.25" customHeight="1">
@@ -7295,9 +7421,10 @@
       <c r="F254" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G254" s="80">
-        <f>HOUR(F254-E254)+MINUTE(F254-E254)/100</f>
-        <v>8.35</v>
+      <c r="G254" s="80" t="inlineStr">
+        <is>
+          <t>8.35</t>
+        </is>
       </c>
     </row>
     <row r="255" spans="1:7" ht="14.25" customHeight="1">
@@ -7319,9 +7446,10 @@
       <c r="F255" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="G255" s="80">
-        <f>HOUR(F255-E255)+MINUTE(F255-E255)/100</f>
-        <v>9.05</v>
+      <c r="G255" s="80" t="inlineStr">
+        <is>
+          <t>9.05</t>
+        </is>
       </c>
     </row>
     <row r="256" spans="1:7" ht="14.25" customHeight="1">
@@ -7779,9 +7907,10 @@
       <c r="F282" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G282" s="80">
-        <f>HOUR(F282-E282)+MINUTE(F282-E282)/100</f>
-        <v>9.07</v>
+      <c r="G282" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="283" spans="1:7" ht="14.25" customHeight="1">
@@ -7803,9 +7932,10 @@
       <c r="F283" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G283" s="80">
-        <f>HOUR(F283-E283)+MINUTE(F283-E283)/100</f>
-        <v>9.1</v>
+      <c r="G283" s="80" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="284" spans="1:7" ht="14.25" customHeight="1">
@@ -7827,9 +7957,10 @@
       <c r="F284" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G284" s="80">
-        <f>HOUR(F284-E284)+MINUTE(F284-E284)/100</f>
-        <v>8.59</v>
+      <c r="G284" s="80" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
       </c>
     </row>
     <row r="285" spans="1:7" ht="14.25" customHeight="1">
@@ -7851,9 +7982,10 @@
       <c r="F285" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="G285" s="80">
-        <f>HOUR(F285-E285)+MINUTE(F285-E285)/100</f>
-        <v>4.47</v>
+      <c r="G285" s="80" t="inlineStr">
+        <is>
+          <t>4.47</t>
+        </is>
       </c>
     </row>
     <row r="286" spans="1:7" ht="14.25" customHeight="1">
@@ -7875,9 +8007,10 @@
       <c r="F286" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G286" s="80">
-        <f>HOUR(F286-E286)+MINUTE(F286-E286)/100</f>
-        <v>9.05</v>
+      <c r="G286" s="80" t="inlineStr">
+        <is>
+          <t>9.05</t>
+        </is>
       </c>
     </row>
     <row r="287" spans="1:7" ht="14.25" customHeight="1">
@@ -7908,9 +8041,10 @@
       <c r="F288" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="G288" s="80">
-        <f>HOUR(F288-E288)+MINUTE(F288-E288)/100</f>
-        <v>9.27</v>
+      <c r="G288" s="80" t="inlineStr">
+        <is>
+          <t>9.27</t>
+        </is>
       </c>
     </row>
     <row r="289" spans="1:7" ht="14.25" customHeight="1">
@@ -7932,9 +8066,10 @@
       <c r="F289" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G289" s="80">
-        <f>HOUR(F289-E289)+MINUTE(F289-E289)/100</f>
-        <v>9.29</v>
+      <c r="G289" s="80" t="inlineStr">
+        <is>
+          <t>9.29</t>
+        </is>
       </c>
     </row>
     <row r="290" spans="1:7" ht="14.25" customHeight="1">
@@ -7956,9 +8091,10 @@
       <c r="F290" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G290" s="80">
-        <f>HOUR(F290-E290)+MINUTE(F290-E290)/100</f>
-        <v>9.02</v>
+      <c r="G290" s="80" t="inlineStr">
+        <is>
+          <t>9.02</t>
+        </is>
       </c>
     </row>
     <row r="291" spans="1:7" ht="14.25" customHeight="1">
@@ -8003,9 +8139,10 @@
       <c r="F292" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G292" s="80">
-        <f>HOUR(F292-E292)+MINUTE(F292-E292)/100</f>
-        <v>9.12</v>
+      <c r="G292" s="80" t="inlineStr">
+        <is>
+          <t>9.12</t>
+        </is>
       </c>
     </row>
     <row r="293" spans="1:7" ht="14.25" customHeight="1">
@@ -8027,9 +8164,10 @@
       <c r="F293" s="29">
         <v>0.71250000000000002</v>
       </c>
-      <c r="G293" s="80">
-        <f>HOUR(F293-E293)+MINUTE(F293-E293)/100</f>
-        <v>9.07</v>
+      <c r="G293" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="294" spans="1:7" ht="14.25" customHeight="1">
@@ -8074,9 +8212,10 @@
       <c r="F295" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G295" s="80">
-        <f>HOUR(F295-E295)+MINUTE(F295-E295)/100</f>
-        <v>9.04</v>
+      <c r="G295" s="80" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
       </c>
     </row>
     <row r="296" spans="1:7" ht="14.25" customHeight="1">
@@ -8098,9 +8237,10 @@
       <c r="F296" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G296" s="80">
-        <f>HOUR(F296-E296)+MINUTE(F296-E296)/100</f>
-        <v>8.58</v>
+      <c r="G296" s="80" t="inlineStr">
+        <is>
+          <t>8.58</t>
+        </is>
       </c>
     </row>
     <row r="297" spans="1:7" ht="14.25" customHeight="1">
@@ -8122,9 +8262,10 @@
       <c r="F297" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G297" s="80">
-        <f>HOUR(F297-E297)+MINUTE(F297-E297)/100</f>
-        <v>9</v>
+      <c r="G297" s="80" t="inlineStr">
+        <is>
+          <t>9.00</t>
+        </is>
       </c>
     </row>
     <row r="298" spans="1:7" ht="14.25" customHeight="1">
@@ -8169,9 +8310,10 @@
       <c r="F299" s="29">
         <v>0.71875</v>
       </c>
-      <c r="G299" s="80">
-        <f>HOUR(F299-E299)+MINUTE(F299-E299)/100</f>
-        <v>9.22</v>
+      <c r="G299" s="80" t="inlineStr">
+        <is>
+          <t>9.22</t>
+        </is>
       </c>
     </row>
     <row r="300" spans="1:7" ht="14.25" customHeight="1">
@@ -8193,9 +8335,10 @@
       <c r="F300" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="G300" s="80">
-        <f>HOUR(F300-E300)+MINUTE(F300-E300)/100</f>
-        <v>9.13</v>
+      <c r="G300" s="80" t="inlineStr">
+        <is>
+          <t>9.13</t>
+        </is>
       </c>
     </row>
     <row r="301" spans="1:7" ht="14.25" customHeight="1">
@@ -8217,9 +8360,10 @@
       <c r="F301" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G301" s="80">
-        <f>HOUR(F301-E301)+MINUTE(F301-E301)/100</f>
-        <v>9.03</v>
+      <c r="G301" s="80" t="inlineStr">
+        <is>
+          <t>9.03</t>
+        </is>
       </c>
     </row>
     <row r="302" spans="1:7" ht="14.25" customHeight="1">
@@ -8241,9 +8385,10 @@
       <c r="F302" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G302" s="80">
-        <f>HOUR(F302-E302)+MINUTE(F302-E302)/100</f>
-        <v>9.1</v>
+      <c r="G302" s="80" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="303" spans="1:7" ht="14.25" customHeight="1">
@@ -8265,9 +8410,10 @@
       <c r="F303" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="G303" s="80">
-        <f>HOUR(F303-E303)+MINUTE(F303-E303)/100</f>
-        <v>9.08</v>
+      <c r="G303" s="80" t="inlineStr">
+        <is>
+          <t>9.08</t>
+        </is>
       </c>
     </row>
     <row r="304" spans="1:7" ht="14.25" customHeight="1">
@@ -8289,9 +8435,10 @@
       <c r="F304" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G304" s="80">
-        <f>HOUR(F304-E304)+MINUTE(F304-E304)/100</f>
-        <v>9.03</v>
+      <c r="G304" s="80" t="inlineStr">
+        <is>
+          <t>9.03</t>
+        </is>
       </c>
     </row>
     <row r="305" spans="1:7" ht="14.25" customHeight="1">
@@ -8336,9 +8483,10 @@
       <c r="F306" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G306" s="80">
-        <f>HOUR(F306-E306)+MINUTE(F306-E306)/100</f>
-        <v>9.07</v>
+      <c r="G306" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="307" spans="1:7" ht="14.25" customHeight="1">
@@ -8360,9 +8508,10 @@
       <c r="F307" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G307" s="80">
-        <f>HOUR(F307-E307)+MINUTE(F307-E307)/100</f>
-        <v>8.59</v>
+      <c r="G307" s="80" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
       </c>
     </row>
     <row r="308" spans="1:7" ht="14.25" customHeight="1">
@@ -8384,9 +8533,10 @@
       <c r="F308" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G308" s="80">
-        <f>HOUR(F308-E308)+MINUTE(F308-E308)/100</f>
-        <v>8.51</v>
+      <c r="G308" s="80" t="inlineStr">
+        <is>
+          <t>8.51</t>
+        </is>
       </c>
     </row>
     <row r="309" spans="1:7" ht="14.25" customHeight="1">
@@ -8408,9 +8558,10 @@
       <c r="F309" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G309" s="80">
-        <f>HOUR(F309-E309)+MINUTE(F309-E309)/100</f>
-        <v>9.01</v>
+      <c r="G309" s="80" t="inlineStr">
+        <is>
+          <t>9.01</t>
+        </is>
       </c>
     </row>
     <row r="310" spans="1:7" ht="14.25" customHeight="1">
@@ -8455,9 +8606,10 @@
       <c r="F311" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G311" s="80">
-        <f>HOUR(F311-E311)+MINUTE(F311-E311)/100</f>
-        <v>8.56</v>
+      <c r="G311" s="80" t="inlineStr">
+        <is>
+          <t>8.56</t>
+        </is>
       </c>
     </row>
     <row r="312" spans="1:7" ht="14.25" customHeight="1">
@@ -8502,9 +8654,10 @@
       <c r="F313" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G313" s="80">
-        <f>HOUR(F313-E313)+MINUTE(F313-E313)/100</f>
-        <v>9.07</v>
+      <c r="G313" s="80" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
       </c>
     </row>
     <row r="314" spans="1:7" ht="14.25" customHeight="1">
@@ -8526,9 +8679,10 @@
       <c r="F314" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="G314" s="80">
-        <f>HOUR(F314-E314)+MINUTE(F314-E314)/100</f>
-        <v>4.51</v>
+      <c r="G314" s="80" t="inlineStr">
+        <is>
+          <t>4.51</t>
+        </is>
       </c>
     </row>
     <row r="315" spans="1:7" ht="14.25" customHeight="1">
@@ -8550,9 +8704,10 @@
       <c r="F315" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G315" s="80">
-        <f>HOUR(F315-E315)+MINUTE(F315-E315)/100</f>
-        <v>8.51</v>
+      <c r="G315" s="80" t="inlineStr">
+        <is>
+          <t>8.51</t>
+        </is>
       </c>
     </row>
     <row r="316" spans="1:7" ht="14.25" customHeight="1">
@@ -8574,9 +8729,10 @@
       <c r="F316" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="G316" s="80">
-        <f>HOUR(F316-E316)+MINUTE(F316-E316)/100</f>
-        <v>8.56</v>
+      <c r="G316" s="80" t="inlineStr">
+        <is>
+          <t>8.56</t>
+        </is>
       </c>
     </row>
     <row r="317" spans="1:7" ht="14.25" customHeight="1">
@@ -8598,9 +8754,10 @@
       <c r="F317" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="G317" s="80">
-        <f>HOUR(F317-E317)+MINUTE(F317-E317)/100</f>
-        <v>9.16</v>
+      <c r="G317" s="80" t="inlineStr">
+        <is>
+          <t>9.16</t>
+        </is>
       </c>
     </row>
     <row r="318" spans="1:7" ht="14.25" customHeight="1">
@@ -8627,9 +8784,10 @@
       <c r="F319" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="G319" s="80">
-        <f>HOUR(F319-E319)+MINUTE(F319-E319)/100</f>
-        <v>7.03</v>
+      <c r="G319" s="80" t="inlineStr">
+        <is>
+          <t>7.03</t>
+        </is>
       </c>
     </row>
     <row r="320" spans="1:7" ht="14.25" customHeight="1">
@@ -8647,9 +8805,10 @@
       <c r="F320" s="75" t="s">
         <v>176</v>
       </c>
-      <c r="G320" s="80">
-        <f>HOUR(F320-E320)+MINUTE(F320-E320)/100</f>
-        <v>9.1</v>
+      <c r="G320" s="80" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
       </c>
     </row>
     <row r="321" spans="1:7" ht="14.25" customHeight="1">
@@ -8724,9 +8883,10 @@
       <c r="F324" s="75" t="s">
         <v>178</v>
       </c>
-      <c r="G324" s="80">
-        <f>HOUR(F324-E324)+MINUTE(F324-E324)/100</f>
-        <v>3.01</v>
+      <c r="G324" s="80" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
       </c>
     </row>
     <row r="325" spans="1:7" ht="14.25" customHeight="1">
@@ -8763,9 +8923,10 @@
       <c r="F326" s="75" t="s">
         <v>179</v>
       </c>
-      <c r="G326" s="80">
-        <f>HOUR(F326-E326)+MINUTE(F326-E326)/100</f>
-        <v>1.07</v>
+      <c r="G326" s="80" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
     </row>
     <row r="327" spans="1:7" ht="14.25" customHeight="1">
@@ -8783,9 +8944,10 @@
       <c r="F327" s="75" t="s">
         <v>180</v>
       </c>
-      <c r="G327" s="80">
-        <f>HOUR(F327-E327)+MINUTE(F327-E327)/100</f>
-        <v>8.44</v>
+      <c r="G327" s="80" t="inlineStr">
+        <is>
+          <t>8.44</t>
+        </is>
       </c>
     </row>
     <row r="328" spans="1:7" ht="14.25" customHeight="1">
@@ -8803,9 +8965,10 @@
       <c r="F328" s="75" t="s">
         <v>181</v>
       </c>
-      <c r="G328" s="80">
-        <f>HOUR(F328-E328)+MINUTE(F328-E328)/100</f>
-        <v>8.34</v>
+      <c r="G328" s="80" t="inlineStr">
+        <is>
+          <t>8.34</t>
+        </is>
       </c>
     </row>
     <row r="329" spans="1:7" ht="14.25" customHeight="1">
@@ -8842,9 +9005,10 @@
       <c r="F330" s="75" t="s">
         <v>165</v>
       </c>
-      <c r="G330" s="80">
-        <f>HOUR(F330-E330)+MINUTE(F330-E330)/100</f>
-        <v>6.06</v>
+      <c r="G330" s="80" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
       </c>
     </row>
     <row r="331" spans="1:7" ht="14.25" customHeight="1">
@@ -8862,9 +9026,10 @@
       <c r="F331" s="75" t="s">
         <v>182</v>
       </c>
-      <c r="G331" s="80">
-        <f>HOUR(F331-E331)+MINUTE(F331-E331)/100</f>
-        <v>8.16</v>
+      <c r="G331" s="80" t="inlineStr">
+        <is>
+          <t>8.16</t>
+        </is>
       </c>
     </row>
     <row r="332" spans="1:7" ht="14.25" customHeight="1">
@@ -8882,9 +9047,10 @@
       <c r="F332" s="75" t="s">
         <v>183</v>
       </c>
-      <c r="G332" s="80">
-        <f>HOUR(F332-E332)+MINUTE(F332-E332)/100</f>
-        <v>7.45</v>
+      <c r="G332" s="80" t="inlineStr">
+        <is>
+          <t>7.45</t>
+        </is>
       </c>
     </row>
     <row r="333" spans="1:7" ht="14.25" customHeight="1">
@@ -8902,9 +9068,10 @@
       <c r="F333" s="75" t="s">
         <v>184</v>
       </c>
-      <c r="G333" s="80">
-        <f>HOUR(F333-E333)+MINUTE(F333-E333)/100</f>
-        <v>7.55</v>
+      <c r="G333" s="80" t="inlineStr">
+        <is>
+          <t>7.55</t>
+        </is>
       </c>
     </row>
     <row r="334" spans="1:7" ht="14.25" customHeight="1">
@@ -8922,9 +9089,10 @@
       <c r="F334" s="75" t="s">
         <v>186</v>
       </c>
-      <c r="G334" s="80">
-        <f>HOUR(F334-E334)+MINUTE(F334-E334)/100</f>
-        <v>4.08</v>
+      <c r="G334" s="80" t="inlineStr">
+        <is>
+          <t>4.08</t>
+        </is>
       </c>
     </row>
     <row r="335" spans="1:7" ht="14.25" customHeight="1">
@@ -8980,9 +9148,10 @@
       <c r="F337" s="75" t="s">
         <v>187</v>
       </c>
-      <c r="G337" s="80">
-        <f>HOUR(F337-E337)+MINUTE(F337-E337)/100</f>
-        <v>4.51</v>
+      <c r="G337" s="80" t="inlineStr">
+        <is>
+          <t>4.51</t>
+        </is>
       </c>
     </row>
     <row r="338" spans="1:7" ht="14.25" customHeight="1">
@@ -9000,9 +9169,10 @@
       <c r="F338" s="75" t="s">
         <v>189</v>
       </c>
-      <c r="G338" s="80">
-        <f>HOUR(F338-E338)+MINUTE(F338-E338)/100</f>
-        <v>0.02</v>
+      <c r="G338" s="80" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
       </c>
     </row>
     <row r="339" spans="1:7" ht="14.25" customHeight="1">
@@ -9153,9 +9323,10 @@
       <c r="F346" s="75" t="s">
         <v>190</v>
       </c>
-      <c r="G346" s="80">
-        <f>HOUR(F346-E346)+MINUTE(F346-E346)/100</f>
-        <v>5.04</v>
+      <c r="G346" s="80" t="inlineStr">
+        <is>
+          <t>5.04</t>
+        </is>
       </c>
     </row>
     <row r="347" spans="1:7" ht="14.25" customHeight="1">
@@ -9224,9 +9395,10 @@
       <c r="F350" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="G350" s="80">
-        <f>HOUR(F350-E350)+MINUTE(F350-E350)/100</f>
-        <v>2.31</v>
+      <c r="G350" s="80" t="inlineStr">
+        <is>
+          <t>2.31</t>
+        </is>
       </c>
     </row>
     <row r="351" spans="1:7" ht="14.25" customHeight="1">
@@ -9432,9 +9604,10 @@
       <c r="F359" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="G359" s="80">
-        <f>HOUR(F359-E359)+MINUTE(F359-E359)/100</f>
-        <v>0.02</v>
+      <c r="G359" s="80" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
       </c>
     </row>
     <row r="360" spans="1:7" ht="14.25" customHeight="1">
@@ -9525,9 +9698,10 @@
       <c r="F363" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="G363" s="80">
-        <f>HOUR(F363-E363)+MINUTE(F363-E363)/100</f>
-        <v>7.53</v>
+      <c r="G363" s="80" t="inlineStr">
+        <is>
+          <t>7.53</t>
+        </is>
       </c>
     </row>
     <row r="364" spans="1:7" ht="14.25" customHeight="1">
@@ -9572,9 +9746,10 @@
       <c r="F365" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="G365" s="80">
-        <f>HOUR(F365-E365)+MINUTE(F365-E365)/100</f>
-        <v>7.21</v>
+      <c r="G365" s="80" t="inlineStr">
+        <is>
+          <t>7.21</t>
+        </is>
       </c>
     </row>
     <row r="366" spans="1:7" ht="14.25" customHeight="1">
@@ -9895,9 +10070,10 @@
       <c r="F379" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="G379" s="80">
-        <f>HOUR(F379-E379)+MINUTE(F379-E379)/100</f>
-        <v>6.52</v>
+      <c r="G379" s="80" t="inlineStr">
+        <is>
+          <t>6.52</t>
+        </is>
       </c>
     </row>
     <row r="380" spans="1:7" ht="14.25" customHeight="1" thickBot="1">

</xml_diff>